<commit_message>
Add reproducibility harness, STROBE checklist, and results polish
(1) run_all.R: one-command staged reproduction (data|analysis|render|all),
defaulting to analysis+render from the committed enriched CSV; heavy/external
steps (Valhalla isochrones, simr power) documented but excluded. Writes a
reproducibility snapshot to repro/ (sessionInfo.txt + package_versions.csv).
(2) manuscript/STROBE_checklist.md: completed 22-item cross-sectional STROBE
checklist mapped to manuscript sections; referenced from the Supplement.
(3) Results polish: report the market-clustering ICC (access 0.043; CBSA log-
scale variance 0.26 for timeliness), translate the significant IRRs into
concrete added wait (~2-3 wk laryngology, ~1-1.5 wk pediatric vs general), and
add a title-page block (keywords, running head, corresponding-author and
word-count placeholders). Verified via a clean full run_all.R pass.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/model_output/supp/supplemental_bundle.xlsx
+++ b/model_output/supp/supplemental_bundle.xlsx
@@ -273,13 +273,13 @@
     <t xml:space="preserve">Date created</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-07-15 21:07:46 MDT</t>
+    <t xml:space="preserve">2026-07-16 21:58:37 MDT</t>
   </si>
   <si>
     <t xml:space="preserve">Package: mysterycall</t>
   </si>
   <si>
-    <t xml:space="preserve">1.6.0.9006</t>
+    <t xml:space="preserve">1.6.0.9010</t>
   </si>
   <si>
     <t xml:space="preserve">Package: openxlsx</t>

</xml_diff>